<commit_message>
Liquidity: graded stress scenarios, collateral-limited borrowing, deposit concentration
- Four default scenarios (as configured, severe, systemic, uninsured run),
  or the settings' Stresses sheet; each through the stressed projection and
  checked against the survival limit.
- A secured contingent line counts at the smaller of its unused amount and
  the lendable value of pledgeable loans (collateral_value) left after
  existing borrowings; secured lines share that headroom.
- depositors.csv gives the uninsured share (new limit uninsured_shares_max)
  and the largest members' share; without it, certificates give a floor.
- Samples: collateral values, secured FHLB lines, synthetic member files;
  the large credit union runs out of liquidity in month 4 under the severe
  scenario. 8 new tests (127 total).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/community-bank/assumptions.xlsx
+++ b/examples/community-bank/assumptions.xlsx
@@ -9,10 +9,11 @@
     <sheet name="Scenarios" sheetId="5" r:id="rId5"/>
     <sheet name="Contingent" sheetId="6" r:id="rId6"/>
     <sheet name="Limits" sheetId="7" r:id="rId7"/>
-    <sheet name="Forecast" sheetId="8" r:id="rId8"/>
-    <sheet name="Drivers" sheetId="9" r:id="rId9"/>
-    <sheet name="Noninterest" sheetId="10" r:id="rId10"/>
-    <sheet name="Notes" sheetId="11" r:id="rId11"/>
+    <sheet name="Stresses" sheetId="8" r:id="rId8"/>
+    <sheet name="Forecast" sheetId="9" r:id="rId9"/>
+    <sheet name="Drivers" sheetId="10" r:id="rId10"/>
+    <sheet name="Noninterest" sheetId="11" r:id="rId11"/>
+    <sheet name="Notes" sheetId="12" r:id="rId12"/>
   </sheets>
 </workbook>
 </file>
@@ -318,6 +319,47 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
+    <col min="1" max="1" width="9" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="4" max="4" width="9" customWidth="1"/>
+    <col min="5" max="5" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">product</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">month</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">volume</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">balance</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">rate</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
     <col min="3" max="3" width="8" customWidth="1"/>
@@ -356,7 +398,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -586,6 +628,7 @@
     <col min="20" max="20" width="16" customWidth="1"/>
     <col min="21" max="21" width="11" customWidth="1"/>
     <col min="22" max="22" width="18" customWidth="1"/>
+    <col min="23" max="23" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -699,6 +742,11 @@
           <t xml:space="preserve">origination_cost</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">collateral_value</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -931,6 +979,9 @@
       <c r="V10">
         <v>0.6</v>
       </c>
+      <c r="W10">
+        <v>60.0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1012,6 +1063,9 @@
       </c>
       <c r="V12">
         <v>1.0</v>
+      </c>
+      <c r="W12">
+        <v>75.0</v>
       </c>
     </row>
     <row r="13">
@@ -1351,6 +1405,7 @@
   <cols>
     <col min="1" max="1" width="54" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1364,6 +1419,11 @@
           <t xml:space="preserve">capacity</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">secured</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1374,6 +1434,9 @@
       <c r="B2">
         <v>117435000.0</v>
       </c>
+      <c r="C2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1383,6 +1446,9 @@
       </c>
       <c r="B3">
         <v>58718000.0</v>
+      </c>
+      <c r="C3" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1567,10 +1633,25 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t xml:space="preserve">uninsured_shares_max</t>
+        </is>
+      </c>
+      <c r="B12">
+        <v>50.0</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Uninsured shares, estimated (at most). Blank uses the default, 15.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t xml:space="preserve">warning_band</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t xml:space="preserve">How close to a limit counts as near it, percent of the limit. Default 10.</t>
         </is>
@@ -1581,6 +1662,53 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="8" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">runoff_multiplier</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">haircut_add</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">contingent_available</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">months</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">uninsured_runoff</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1607,45 +1735,4 @@
     </row>
   </sheetData>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <cols>
-    <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="8" customWidth="1"/>
-    <col min="3" max="3" width="8" customWidth="1"/>
-    <col min="4" max="4" width="9" customWidth="1"/>
-    <col min="5" max="5" width="8" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">product</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">month</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">volume</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">balance</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">rate</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Budget actuals straight from the general ledger's monthly trial balance
trial_balance.csv plus gl_map.csv (account -> line, measure: balance,
activity or ytd) replace a hand-built actuals.csv: natural signs turned
around by line, year-to-date differenced and restarted at the new
fiscal_year_start setting, averages from month-ends. The variance and the
NII back-test read either source; the analysis-date month ties to the
positions in the reconciliation. mid-cu's sample now ships a trial balance
that reproduces its old actuals to the cent.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/community-bank/assumptions.xlsx
+++ b/examples/community-bank/assumptions.xlsx
@@ -9,11 +9,12 @@
     <sheet name="Scenarios" sheetId="5" r:id="rId5"/>
     <sheet name="Contingent" sheetId="6" r:id="rId6"/>
     <sheet name="Limits" sheetId="7" r:id="rId7"/>
-    <sheet name="Stresses" sheetId="8" r:id="rId8"/>
-    <sheet name="Forecast" sheetId="9" r:id="rId9"/>
-    <sheet name="Drivers" sheetId="10" r:id="rId10"/>
-    <sheet name="Noninterest" sheetId="11" r:id="rId11"/>
-    <sheet name="Notes" sheetId="12" r:id="rId12"/>
+    <sheet name="CreditScenarios" sheetId="8" r:id="rId8"/>
+    <sheet name="Stresses" sheetId="9" r:id="rId9"/>
+    <sheet name="Forecast" sheetId="10" r:id="rId10"/>
+    <sheet name="Drivers" sheetId="11" r:id="rId11"/>
+    <sheet name="Noninterest" sheetId="12" r:id="rId12"/>
+    <sheet name="Notes" sheetId="13" r:id="rId13"/>
   </sheets>
 </workbook>
 </file>
@@ -319,6 +320,35 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">month</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">tenor_months</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">rate</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
     <col min="3" max="3" width="8" customWidth="1"/>
@@ -357,7 +387,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -398,7 +428,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1665,6 +1695,41 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">multiplier</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">months</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">reversion_months</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
@@ -1706,33 +1771,4 @@
     </row>
   </sheetData>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <cols>
-    <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="8" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">month</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">tenor_months</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">rate</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Basis risk, separate index curves, and a prepayment model
Indexes can have their own curve and a beta to the main curve; scenarios
can carry a basis (per index, or 'shares' for administered rates), in the
settings' Indexes and Scenarios sheets. The rate-risk section adds a
basis-risk table (each index +/-50bp and share rates +/-25bp against the
curve, alone) and a finding. Products can run a prepayment model: speed
from each loan's own refinancing incentive, burnout over months in the
money, and seasoning from loan age, which the importer now carries on
pools. large-cu's mortgages use it, with a prime-lags scenario. Defaults
leave every existing result unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/community-bank/assumptions.xlsx
+++ b/examples/community-bank/assumptions.xlsx
@@ -584,6 +584,8 @@
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="4" max="4" width="8" customWidth="1"/>
+    <col min="5" max="5" width="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -600,6 +602,16 @@
       <c r="C1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">spread</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">beta</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">curve</t>
         </is>
       </c>
     </row>
@@ -1352,6 +1364,7 @@
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1373,6 +1386,11 @@
       <c r="D1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">shape</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">basis</t>
         </is>
       </c>
     </row>

</xml_diff>